<commit_message>
Use regular prices instead of new-shopper promo prices
aliexpress.com search shows a first-order price when a listing says
"New shoppers save $X". Kit and other .com prices now use the regular
price (shown + X): CaDA, Rastar and replica kits cost 2-3x more than
the first report said. Regenerate the listing CSV and models list,
fix the research report tables and the assortment workbook.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VJZmy9D7cUuAqNKujKfv3T
</commit_message>
<xml_diff>
--- a/f1-shop/data/tmff-assortment.xlsx
+++ b/f1-shop/data/tmff-assortment.xlsx
@@ -41,7 +41,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Цена из выдачи aliexpress.com в $, пересчитана по курсу 84,2 ₽/$ (лист «Параметры»).</t>
+          <t xml:space="preserve">Обычная цена из выдачи aliexpress.com (без скидки для новых покупателей), пересчитана из $ по курсу 84,2 ₽/$.</t>
         </r>
       </text>
     </comment>
@@ -53,7 +53,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Цена из выдачи aliexpress.com в $, пересчитана по курсу 84,2 ₽/$ (лист «Параметры»).</t>
+          <t xml:space="preserve">Обычная цена из выдачи aliexpress.com (без скидки для новых покупателей), пересчитана из $ по курсу 84,2 ₽/$.</t>
         </r>
       </text>
     </comment>
@@ -65,7 +65,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Цена из выдачи aliexpress.com в $, пересчитана по курсу 84,2 ₽/$ (лист «Параметры»).</t>
+          <t xml:space="preserve">Обычная цена из выдачи aliexpress.com (без скидки для новых покупателей), пересчитана из $ по курсу 84,2 ₽/$.</t>
         </r>
       </text>
     </comment>
@@ -77,7 +77,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Цена из выдачи aliexpress.com в $, пересчитана по курсу 84,2 ₽/$ (лист «Параметры»).</t>
+          <t xml:space="preserve">Обычная цена из выдачи aliexpress.com (без скидки для новых покупателей), пересчитана из $ по курсу 84,2 ₽/$.</t>
         </r>
       </text>
     </comment>
@@ -89,7 +89,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Цена из выдачи aliexpress.com в $, пересчитана по курсу 84,2 ₽/$ (лист «Параметры»).</t>
+          <t xml:space="preserve">Обычная цена из выдачи aliexpress.com (без скидки для новых покупателей), пересчитана из $ по курсу 84,2 ₽/$.</t>
         </r>
       </text>
     </comment>
@@ -101,7 +101,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Цена из выдачи aliexpress.com в $, пересчитана по курсу 84,2 ₽/$ (лист «Параметры»).</t>
+          <t xml:space="preserve">Обычная цена из выдачи aliexpress.com (без скидки для новых покупателей), пересчитана из $ по курсу 84,2 ₽/$.</t>
         </r>
       </text>
     </comment>
@@ -113,7 +113,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Цена из выдачи aliexpress.com в $, пересчитана по курсу 84,2 ₽/$ (лист «Параметры»).</t>
+          <t xml:space="preserve">Обычная цена из выдачи aliexpress.com (без скидки для новых покупателей), пересчитана из $ по курсу 84,2 ₽/$.</t>
         </r>
       </text>
     </comment>
@@ -125,7 +125,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Цена из выдачи aliexpress.com в $, пересчитана по курсу 84,2 ₽/$ (лист «Параметры»).</t>
+          <t xml:space="preserve">Обычная цена из выдачи aliexpress.com (без скидки для новых покупателей), пересчитана из $ по курсу 84,2 ₽/$.</t>
         </r>
       </text>
     </comment>
@@ -137,7 +137,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Цена из выдачи aliexpress.com в $, пересчитана по курсу 84,2 ₽/$ (лист «Параметры»).</t>
+          <t xml:space="preserve">Обычная цена из выдачи aliexpress.com (без скидки для новых покупателей), пересчитана из $ по курсу 84,2 ₽/$.</t>
         </r>
       </text>
     </comment>
@@ -149,7 +149,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Цена из выдачи aliexpress.com в $, пересчитана по курсу 84,2 ₽/$ (лист «Параметры»).</t>
+          <t xml:space="preserve">Обычная цена из выдачи aliexpress.com (без скидки для новых покупателей), пересчитана из $ по курсу 84,2 ₽/$.</t>
         </r>
       </text>
     </comment>
@@ -158,12 +158,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1223" uniqueCount="367">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1226" uniqueCount="368">
   <si>
     <t xml:space="preserve">TMFF — стартовый ассортимент</t>
   </si>
   <si>
-    <t xml:space="preserve">Синим — данные AliExpress (варианты лотов собраны в Chrome 25.09.2026, конструкторы — из поиска aliexpress.com), чёрным — формулы, жёлтым — проверить. Цена — за товар, без платной доставки, если она есть.</t>
+    <t xml:space="preserve">Синим — данные AliExpress (варианты лотов собраны в Chrome 25.09.2026, конструкторы — из поиска aliexpress.com), чёрным — формулы, жёлтым — проверить. Цена — за товар, без платной доставки, если она есть. У конструкторов — обычная цена, без скидки для новых покупателей.</t>
   </si>
   <si>
     <t xml:space="preserve">Повторы убраны: болид + пилот + ливрея + масштаб встречаются один раз, по самой низкой цене. Другие лоты с тем же вариантом — в «Запасной лот». «Вариант на Ali» — что выбрать при заказе.</t>
@@ -628,7 +628,7 @@
     <t xml:space="preserve">проверить</t>
   </si>
   <si>
-    <t xml:space="preserve">Официальная лицензия Alpine. Цена из $ по курсу. Вариант «с коробкой» и его цену не проверяли: в CSV из Chrome этого лота нет.</t>
+    <t xml:space="preserve">Официальная лицензия Alpine. Вариант «с коробкой» и его цену не проверяли: в CSV из Chrome этого лота нет.</t>
   </si>
   <si>
     <t xml:space="preserve">CaDA Kick Sauber C44</t>
@@ -658,7 +658,10 @@
     <t xml:space="preserve">реплика</t>
   </si>
   <si>
-    <t xml:space="preserve">Лот с вариантами SF-24 / RB20. Запасной продавец: 3256812748054401 · 1 636 ₽, оценка 4.7. Вариант «с коробкой» и его цену не проверяли: в CSV из Chrome этого лота нет.</t>
+    <t xml:space="preserve">796303924 · 5 118 ₽, оценка 4.9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Лот с вариантами SF-24 / RB20. Вариант «с коробкой» и его цену не проверяли: в CSV из Chrome этого лота нет.</t>
   </si>
   <si>
     <t xml:space="preserve">Red Bull RB20, 1 639 деталей — реплика</t>
@@ -670,7 +673,7 @@
     <t xml:space="preserve">McLaren MCL39, 1 675 деталей — реплика</t>
   </si>
   <si>
-    <t xml:space="preserve">В лоте есть и SF-24 / RB20 — брать только MCL39. Вариант «с коробкой» и его цену не проверяли: в CSV из Chrome этого лота нет.</t>
+    <t xml:space="preserve">В лоте есть и SF-24 / RB20 — брать только MCL39. Цена в выдаче — возможно, другого варианта: сверить. Вариант «с коробкой» и его цену не проверяли: в CSV из Chrome этого лота нет.</t>
   </si>
   <si>
     <t xml:space="preserve">Mercedes W14 E, 1 642 детали — реплика</t>
@@ -691,15 +694,15 @@
     <t xml:space="preserve">Red Bull RB21 — Mould King MK6025</t>
   </si>
   <si>
-    <t xml:space="preserve">Свой дизайн Mould King, ливрея без лицензии. Запасной продавец: 3256812310056041 · 4 699 ₽. Вариант «с коробкой» и его цену не проверяли: в CSV из Chrome этого лота нет.</t>
+    <t xml:space="preserve">605226634 · 5 708 ₽, оценка 4.8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Свой дизайн Mould King, ливрея без лицензии. Вариант «с коробкой» и его цену не проверяли: в CSV из Chrome этого лота нет.</t>
   </si>
   <si>
     <t xml:space="preserve">Aston Martin AMR25 — Mould King MK6022</t>
   </si>
   <si>
-    <t xml:space="preserve">Свой дизайн Mould King, ливрея без лицензии. Вариант «с коробкой» и его цену не проверяли: в CSV из Chrome этого лота нет.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Постеры</t>
   </si>
   <si>
@@ -1201,7 +1204,7 @@
     <t xml:space="preserve">Конструкторы CaDA (3 лота)</t>
   </si>
   <si>
-    <t xml:space="preserve">Цена нужного варианта и есть ли коробка. У C44 1:8 — что это набор C64010W на 2 553 детали. В CSV из Chrome этих лотов нет, цены — из поиска aliexpress.com.</t>
+    <t xml:space="preserve">Цена нужного варианта и есть ли коробка. У C44 1:8 — что это набор C64010W на 2 553 детали. В CSV из Chrome этих лотов нет, цены — из поиска aliexpress.com: там показана цена для новых покупателей, в таблице — обычная (в 2–3 раза выше).</t>
   </si>
   <si>
     <t xml:space="preserve">Реплики конструкторов (7 лотов)</t>
@@ -1564,7 +1567,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="8">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1608,6 +1611,14 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FF0563C1"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF4CCCC"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -4111,15 +4122,15 @@
         <v>109</v>
       </c>
       <c r="D42" s="7" t="n">
-        <v>1588</v>
+        <v>4524</v>
       </c>
       <c r="E42" s="8" t="n">
         <f aca="false">IF(D42="","",IF(D42&lt;Параметры!$B$4,CEILING(D42*Параметры!$B$5,100)-10,IF(D42&lt;=Параметры!$B$6,CEILING(D42*Параметры!$B$7,100)-10,CEILING(D42*Параметры!$B$8,100)-10)))</f>
-        <v>2590</v>
+        <v>7290</v>
       </c>
       <c r="F42" s="8" t="n">
         <f aca="false">IF(D42="","",ROUND(E42*(1-Параметры!$B$9-Параметры!$B$10-Параметры!$B$11)-D42,0))</f>
-        <v>626</v>
+        <v>1709</v>
       </c>
       <c r="G42" s="9" t="s">
         <v>87</v>
@@ -4152,7 +4163,7 @@
       </c>
       <c r="Q42" s="9" t="str">
         <f aca="false">IF(C42&lt;&gt;"1:24","",IF(D42="","проверить",IF(D42&lt;=Параметры!$B$12,"ок","дороже лимита")))</f>
-        <v>ок</v>
+        <v>дороже лимита</v>
       </c>
       <c r="R42" s="14" t="s">
         <v>156</v>
@@ -4169,15 +4180,15 @@
         <v>109</v>
       </c>
       <c r="D43" s="7" t="n">
-        <v>1822</v>
+        <v>6648</v>
       </c>
       <c r="E43" s="8" t="n">
         <f aca="false">IF(D43="","",IF(D43&lt;Параметры!$B$4,CEILING(D43*Параметры!$B$5,100)-10,IF(D43&lt;=Параметры!$B$6,CEILING(D43*Параметры!$B$7,100)-10,CEILING(D43*Параметры!$B$8,100)-10)))</f>
-        <v>2990</v>
+        <v>10690</v>
       </c>
       <c r="F43" s="8" t="n">
         <f aca="false">IF(D43="","",ROUND(E43*(1-Параметры!$B$9-Параметры!$B$10-Параметры!$B$11)-D43,0))</f>
-        <v>734</v>
+        <v>2492</v>
       </c>
       <c r="G43" s="9" t="s">
         <v>158</v>
@@ -4210,7 +4221,7 @@
       </c>
       <c r="Q43" s="9" t="str">
         <f aca="false">IF(C43&lt;&gt;"1:24","",IF(D43="","проверить",IF(D43&lt;=Параметры!$B$12,"ок","дороже лимита")))</f>
-        <v>ок</v>
+        <v>дороже лимита</v>
       </c>
       <c r="R43" s="14" t="s">
         <v>159</v>
@@ -4227,15 +4238,15 @@
         <v>161</v>
       </c>
       <c r="D44" s="7" t="n">
-        <v>10614</v>
+        <v>25084</v>
       </c>
       <c r="E44" s="8" t="n">
         <f aca="false">IF(D44="","",IF(D44&lt;Параметры!$B$4,CEILING(D44*Параметры!$B$5,100)-10,IF(D44&lt;=Параметры!$B$6,CEILING(D44*Параметры!$B$7,100)-10,CEILING(D44*Параметры!$B$8,100)-10)))</f>
-        <v>14390</v>
+        <v>33890</v>
       </c>
       <c r="F44" s="8" t="n">
         <f aca="false">IF(D44="","",ROUND(E44*(1-Параметры!$B$9-Параметры!$B$10-Параметры!$B$11)-D44,0))</f>
-        <v>1689</v>
+        <v>3892</v>
       </c>
       <c r="G44" s="9" t="s">
         <v>158</v>
@@ -4285,15 +4296,15 @@
         <v>161</v>
       </c>
       <c r="D45" s="7" t="n">
-        <v>1747</v>
+        <v>4866</v>
       </c>
       <c r="E45" s="8" t="n">
         <f aca="false">IF(D45="","",IF(D45&lt;Параметры!$B$4,CEILING(D45*Параметры!$B$5,100)-10,IF(D45&lt;=Параметры!$B$6,CEILING(D45*Параметры!$B$7,100)-10,CEILING(D45*Параметры!$B$8,100)-10)))</f>
-        <v>2790</v>
+        <v>7790</v>
       </c>
       <c r="F45" s="8" t="n">
         <f aca="false">IF(D45="","",ROUND(E45*(1-Параметры!$B$9-Параметры!$B$10-Параметры!$B$11)-D45,0))</f>
-        <v>638</v>
+        <v>1794</v>
       </c>
       <c r="G45" s="9" t="s">
         <v>123</v>
@@ -4311,7 +4322,7 @@
         <v>1000</v>
       </c>
       <c r="L45" s="11" t="n">
-        <v>4.9</v>
+        <v>4.7</v>
       </c>
       <c r="M45" s="12" t="s">
         <v>27</v>
@@ -4319,7 +4330,9 @@
       <c r="N45" s="15" t="s">
         <v>155</v>
       </c>
-      <c r="O45" s="13"/>
+      <c r="O45" s="13" t="s">
+        <v>166</v>
+      </c>
       <c r="P45" s="9" t="str">
         <f aca="false">IF(COUNTIFS($G$5:$G$72,G45,$H$5:$H$72,H45,$I$5:$I$72,I45,$C$5:$C$72,C45)&gt;1,"повтор","")</f>
         <v/>
@@ -4329,7 +4342,7 @@
         <v/>
       </c>
       <c r="R45" s="14" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4337,21 +4350,21 @@
         <v>163</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C46" s="6" t="s">
         <v>161</v>
       </c>
       <c r="D46" s="7" t="n">
-        <v>1747</v>
+        <v>4866</v>
       </c>
       <c r="E46" s="8" t="n">
         <f aca="false">IF(D46="","",IF(D46&lt;Параметры!$B$4,CEILING(D46*Параметры!$B$5,100)-10,IF(D46&lt;=Параметры!$B$6,CEILING(D46*Параметры!$B$7,100)-10,CEILING(D46*Параметры!$B$8,100)-10)))</f>
-        <v>2790</v>
+        <v>7790</v>
       </c>
       <c r="F46" s="8" t="n">
         <f aca="false">IF(D46="","",ROUND(E46*(1-Параметры!$B$9-Параметры!$B$10-Параметры!$B$11)-D46,0))</f>
-        <v>638</v>
+        <v>1794</v>
       </c>
       <c r="G46" s="9" t="s">
         <v>115</v>
@@ -4369,7 +4382,7 @@
         <v>1000</v>
       </c>
       <c r="L46" s="11" t="n">
-        <v>4.9</v>
+        <v>4.7</v>
       </c>
       <c r="M46" s="12" t="s">
         <v>27</v>
@@ -4377,7 +4390,9 @@
       <c r="N46" s="15" t="s">
         <v>155</v>
       </c>
-      <c r="O46" s="13"/>
+      <c r="O46" s="13" t="s">
+        <v>166</v>
+      </c>
       <c r="P46" s="9" t="str">
         <f aca="false">IF(COUNTIFS($G$5:$G$72,G46,$H$5:$H$72,H46,$I$5:$I$72,I46,$C$5:$C$72,C46)&gt;1,"повтор","")</f>
         <v/>
@@ -4387,7 +4402,7 @@
         <v/>
       </c>
       <c r="R46" s="14" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4395,7 +4410,7 @@
         <v>163</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C47" s="6" t="s">
         <v>161</v>
@@ -4445,7 +4460,7 @@
         <v/>
       </c>
       <c r="R47" s="14" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4453,24 +4468,24 @@
         <v>163</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C48" s="6" t="s">
         <v>161</v>
       </c>
       <c r="D48" s="7" t="n">
-        <v>1423</v>
+        <v>4383</v>
       </c>
       <c r="E48" s="8" t="n">
         <f aca="false">IF(D48="","",IF(D48&lt;Параметры!$B$4,CEILING(D48*Параметры!$B$5,100)-10,IF(D48&lt;=Параметры!$B$6,CEILING(D48*Параметры!$B$7,100)-10,CEILING(D48*Параметры!$B$8,100)-10)))</f>
-        <v>2890</v>
+        <v>7090</v>
       </c>
       <c r="F48" s="8" t="n">
         <f aca="false">IF(D48="","",ROUND(E48*(1-Параметры!$B$9-Параметры!$B$10-Параметры!$B$11)-D48,0))</f>
-        <v>1048</v>
+        <v>1679</v>
       </c>
       <c r="G48" s="9" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="H48" s="9" t="s">
         <v>153</v>
@@ -4501,7 +4516,7 @@
         <v/>
       </c>
       <c r="R48" s="14" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4509,21 +4524,21 @@
         <v>163</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C49" s="6" t="s">
         <v>161</v>
       </c>
       <c r="D49" s="7" t="n">
-        <v>2180</v>
+        <v>5967</v>
       </c>
       <c r="E49" s="8" t="n">
         <f aca="false">IF(D49="","",IF(D49&lt;Параметры!$B$4,CEILING(D49*Параметры!$B$5,100)-10,IF(D49&lt;=Параметры!$B$6,CEILING(D49*Параметры!$B$7,100)-10,CEILING(D49*Параметры!$B$8,100)-10)))</f>
-        <v>3490</v>
+        <v>9590</v>
       </c>
       <c r="F49" s="8" t="n">
         <f aca="false">IF(D49="","",ROUND(E49*(1-Параметры!$B$9-Параметры!$B$10-Параметры!$B$11)-D49,0))</f>
-        <v>804</v>
+        <v>2232</v>
       </c>
       <c r="G49" s="9" t="s">
         <v>41</v>
@@ -4559,7 +4574,7 @@
         <v/>
       </c>
       <c r="R49" s="14" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4567,21 +4582,21 @@
         <v>163</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C50" s="6" t="s">
         <v>161</v>
       </c>
       <c r="D50" s="7" t="n">
-        <v>2006</v>
+        <v>4699</v>
       </c>
       <c r="E50" s="8" t="n">
         <f aca="false">IF(D50="","",IF(D50&lt;Параметры!$B$4,CEILING(D50*Параметры!$B$5,100)-10,IF(D50&lt;=Параметры!$B$6,CEILING(D50*Параметры!$B$7,100)-10,CEILING(D50*Параметры!$B$8,100)-10)))</f>
-        <v>3290</v>
+        <v>7590</v>
       </c>
       <c r="F50" s="8" t="n">
         <f aca="false">IF(D50="","",ROUND(E50*(1-Параметры!$B$9-Параметры!$B$10-Параметры!$B$11)-D50,0))</f>
-        <v>807</v>
+        <v>1790</v>
       </c>
       <c r="G50" s="9" t="s">
         <v>24</v>
@@ -4595,11 +4610,11 @@
       <c r="J50" s="9" t="n">
         <v>2025</v>
       </c>
-      <c r="K50" s="16" t="n">
-        <v>1000</v>
+      <c r="K50" s="7" t="n">
+        <v>900</v>
       </c>
       <c r="L50" s="11" t="n">
-        <v>4.8</v>
+        <v>4.7</v>
       </c>
       <c r="M50" s="12" t="s">
         <v>27</v>
@@ -4607,7 +4622,9 @@
       <c r="N50" s="15" t="s">
         <v>155</v>
       </c>
-      <c r="O50" s="13"/>
+      <c r="O50" s="13" t="s">
+        <v>178</v>
+      </c>
       <c r="P50" s="9" t="str">
         <f aca="false">IF(COUNTIFS($G$5:$G$72,G50,$H$5:$H$72,H50,$I$5:$I$72,I50,$C$5:$C$72,C50)&gt;1,"повтор","")</f>
         <v/>
@@ -4617,7 +4634,7 @@
         <v/>
       </c>
       <c r="R50" s="14" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4625,21 +4642,21 @@
         <v>163</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="C51" s="6" t="s">
         <v>161</v>
       </c>
       <c r="D51" s="7" t="n">
-        <v>1904</v>
+        <v>5474</v>
       </c>
       <c r="E51" s="8" t="n">
         <f aca="false">IF(D51="","",IF(D51&lt;Параметры!$B$4,CEILING(D51*Параметры!$B$5,100)-10,IF(D51&lt;=Параметры!$B$6,CEILING(D51*Параметры!$B$7,100)-10,CEILING(D51*Параметры!$B$8,100)-10)))</f>
-        <v>3090</v>
+        <v>8790</v>
       </c>
       <c r="F51" s="8" t="n">
         <f aca="false">IF(D51="","",ROUND(E51*(1-Параметры!$B$9-Параметры!$B$10-Параметры!$B$11)-D51,0))</f>
-        <v>738</v>
+        <v>2041</v>
       </c>
       <c r="G51" s="9" t="s">
         <v>80</v>
@@ -4678,13 +4695,13 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="4" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D52" s="7" t="n">
         <v>629</v>
@@ -4698,7 +4715,7 @@
         <v>474</v>
       </c>
       <c r="G52" s="9" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="H52" s="9" t="s">
         <v>153</v>
@@ -4719,7 +4736,7 @@
         <v>27</v>
       </c>
       <c r="N52" s="6" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="O52" s="13"/>
       <c r="P52" s="9" t="str">
@@ -4731,18 +4748,18 @@
         <v/>
       </c>
       <c r="R52" s="14" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="4" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D53" s="7" t="n">
         <v>629</v>
@@ -4756,7 +4773,7 @@
         <v>474</v>
       </c>
       <c r="G53" s="9" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="H53" s="9" t="s">
         <v>153</v>
@@ -4777,7 +4794,7 @@
         <v>27</v>
       </c>
       <c r="N53" s="6" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="O53" s="13"/>
       <c r="P53" s="9" t="str">
@@ -4789,18 +4806,18 @@
         <v/>
       </c>
       <c r="R53" s="14" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="4" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D54" s="7" t="n">
         <v>629</v>
@@ -4814,7 +4831,7 @@
         <v>474</v>
       </c>
       <c r="G54" s="9" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="H54" s="9" t="s">
         <v>153</v>
@@ -4835,7 +4852,7 @@
         <v>27</v>
       </c>
       <c r="N54" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="O54" s="13"/>
       <c r="P54" s="9" t="str">
@@ -4847,18 +4864,18 @@
         <v/>
       </c>
       <c r="R54" s="14" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="4" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D55" s="7" t="n">
         <v>629</v>
@@ -4872,7 +4889,7 @@
         <v>474</v>
       </c>
       <c r="G55" s="9" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="H55" s="9" t="s">
         <v>153</v>
@@ -4893,7 +4910,7 @@
         <v>27</v>
       </c>
       <c r="N55" s="6" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="O55" s="13"/>
       <c r="P55" s="9" t="str">
@@ -4905,18 +4922,18 @@
         <v/>
       </c>
       <c r="R55" s="14" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="4" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B56" s="5" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D56" s="7" t="n">
         <v>629</v>
@@ -4930,7 +4947,7 @@
         <v>474</v>
       </c>
       <c r="G56" s="9" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="H56" s="9" t="s">
         <v>153</v>
@@ -4951,7 +4968,7 @@
         <v>27</v>
       </c>
       <c r="N56" s="6" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="O56" s="13"/>
       <c r="P56" s="9" t="str">
@@ -4963,18 +4980,18 @@
         <v/>
       </c>
       <c r="R56" s="14" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="4" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B57" s="5" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D57" s="7" t="n">
         <v>629</v>
@@ -4988,7 +5005,7 @@
         <v>474</v>
       </c>
       <c r="G57" s="9" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="H57" s="9" t="s">
         <v>153</v>
@@ -5009,7 +5026,7 @@
         <v>27</v>
       </c>
       <c r="N57" s="6" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="O57" s="13"/>
       <c r="P57" s="9" t="str">
@@ -5021,18 +5038,18 @@
         <v/>
       </c>
       <c r="R57" s="14" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="4" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B58" s="5" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D58" s="7" t="n">
         <v>629</v>
@@ -5046,7 +5063,7 @@
         <v>474</v>
       </c>
       <c r="G58" s="9" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H58" s="9" t="s">
         <v>153</v>
@@ -5067,7 +5084,7 @@
         <v>27</v>
       </c>
       <c r="N58" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="O58" s="13"/>
       <c r="P58" s="9" t="str">
@@ -5079,18 +5096,18 @@
         <v/>
       </c>
       <c r="R58" s="14" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="4" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D59" s="7" t="n">
         <v>629</v>
@@ -5104,7 +5121,7 @@
         <v>474</v>
       </c>
       <c r="G59" s="9" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="H59" s="9" t="s">
         <v>153</v>
@@ -5125,7 +5142,7 @@
         <v>27</v>
       </c>
       <c r="N59" s="6" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="O59" s="13"/>
       <c r="P59" s="9" t="str">
@@ -5137,18 +5154,18 @@
         <v/>
       </c>
       <c r="R59" s="14" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="4" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B60" s="5" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D60" s="7" t="n">
         <v>629</v>
@@ -5162,7 +5179,7 @@
         <v>474</v>
       </c>
       <c r="G60" s="9" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H60" s="9" t="s">
         <v>153</v>
@@ -5183,7 +5200,7 @@
         <v>27</v>
       </c>
       <c r="N60" s="6" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="O60" s="13"/>
       <c r="P60" s="9" t="str">
@@ -5195,18 +5212,18 @@
         <v/>
       </c>
       <c r="R60" s="14" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="4" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B61" s="5" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D61" s="7" t="n">
         <v>629</v>
@@ -5220,7 +5237,7 @@
         <v>474</v>
       </c>
       <c r="G61" s="9" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="H61" s="9" t="s">
         <v>153</v>
@@ -5241,7 +5258,7 @@
         <v>27</v>
       </c>
       <c r="N61" s="6" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="O61" s="13"/>
       <c r="P61" s="9" t="str">
@@ -5253,18 +5270,18 @@
         <v/>
       </c>
       <c r="R61" s="14" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="4" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B62" s="5" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C62" s="6" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D62" s="7" t="n">
         <v>629</v>
@@ -5278,7 +5295,7 @@
         <v>474</v>
       </c>
       <c r="G62" s="9" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="H62" s="9" t="s">
         <v>153</v>
@@ -5299,7 +5316,7 @@
         <v>27</v>
       </c>
       <c r="N62" s="6" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="O62" s="13"/>
       <c r="P62" s="9" t="str">
@@ -5311,18 +5328,18 @@
         <v/>
       </c>
       <c r="R62" s="14" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="4" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B63" s="5" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D63" s="7" t="n">
         <v>629</v>
@@ -5336,7 +5353,7 @@
         <v>474</v>
       </c>
       <c r="G63" s="9" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="H63" s="9" t="s">
         <v>153</v>
@@ -5357,7 +5374,7 @@
         <v>27</v>
       </c>
       <c r="N63" s="6" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="O63" s="13"/>
       <c r="P63" s="9" t="str">
@@ -5369,18 +5386,18 @@
         <v/>
       </c>
       <c r="R63" s="14" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="4" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B64" s="5" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D64" s="7" t="n">
         <v>629</v>
@@ -5394,7 +5411,7 @@
         <v>474</v>
       </c>
       <c r="G64" s="9" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="H64" s="9" t="s">
         <v>153</v>
@@ -5415,7 +5432,7 @@
         <v>27</v>
       </c>
       <c r="N64" s="6" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="O64" s="13"/>
       <c r="P64" s="9" t="str">
@@ -5427,18 +5444,18 @@
         <v/>
       </c>
       <c r="R64" s="14" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="4" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B65" s="5" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C65" s="6" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D65" s="7" t="n">
         <v>629</v>
@@ -5452,7 +5469,7 @@
         <v>474</v>
       </c>
       <c r="G65" s="9" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="H65" s="9" t="s">
         <v>153</v>
@@ -5473,7 +5490,7 @@
         <v>27</v>
       </c>
       <c r="N65" s="6" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="O65" s="13"/>
       <c r="P65" s="9" t="str">
@@ -5485,18 +5502,18 @@
         <v/>
       </c>
       <c r="R65" s="14" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="4" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B66" s="5" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C66" s="6" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D66" s="7" t="n">
         <v>629</v>
@@ -5510,7 +5527,7 @@
         <v>474</v>
       </c>
       <c r="G66" s="9" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="H66" s="9" t="s">
         <v>153</v>
@@ -5531,7 +5548,7 @@
         <v>27</v>
       </c>
       <c r="N66" s="6" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="O66" s="13"/>
       <c r="P66" s="9" t="str">
@@ -5543,18 +5560,18 @@
         <v/>
       </c>
       <c r="R66" s="14" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="4" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B67" s="5" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C67" s="6" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D67" s="7" t="n">
         <v>629</v>
@@ -5568,7 +5585,7 @@
         <v>474</v>
       </c>
       <c r="G67" s="9" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="H67" s="9" t="s">
         <v>153</v>
@@ -5589,7 +5606,7 @@
         <v>27</v>
       </c>
       <c r="N67" s="6" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="O67" s="13"/>
       <c r="P67" s="9" t="str">
@@ -5601,18 +5618,18 @@
         <v/>
       </c>
       <c r="R67" s="14" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="4" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B68" s="5" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C68" s="6" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D68" s="7" t="n">
         <v>629</v>
@@ -5626,7 +5643,7 @@
         <v>474</v>
       </c>
       <c r="G68" s="9" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="H68" s="9" t="s">
         <v>153</v>
@@ -5647,7 +5664,7 @@
         <v>27</v>
       </c>
       <c r="N68" s="6" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="O68" s="13"/>
       <c r="P68" s="9" t="str">
@@ -5659,18 +5676,18 @@
         <v/>
       </c>
       <c r="R68" s="14" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="4" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B69" s="5" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C69" s="6" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D69" s="7" t="n">
         <v>629</v>
@@ -5684,7 +5701,7 @@
         <v>474</v>
       </c>
       <c r="G69" s="9" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="H69" s="9" t="s">
         <v>153</v>
@@ -5705,7 +5722,7 @@
         <v>27</v>
       </c>
       <c r="N69" s="6" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="O69" s="13"/>
       <c r="P69" s="9" t="str">
@@ -5717,18 +5734,18 @@
         <v/>
       </c>
       <c r="R69" s="14" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="4" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B70" s="5" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C70" s="6" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D70" s="7" t="n">
         <v>629</v>
@@ -5742,7 +5759,7 @@
         <v>474</v>
       </c>
       <c r="G70" s="9" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="H70" s="9" t="s">
         <v>153</v>
@@ -5763,7 +5780,7 @@
         <v>27</v>
       </c>
       <c r="N70" s="6" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="O70" s="13"/>
       <c r="P70" s="9" t="str">
@@ -5775,18 +5792,18 @@
         <v/>
       </c>
       <c r="R70" s="14" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="4" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B71" s="5" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C71" s="6" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D71" s="7" t="n">
         <v>629</v>
@@ -5800,7 +5817,7 @@
         <v>474</v>
       </c>
       <c r="G71" s="9" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="H71" s="9" t="s">
         <v>153</v>
@@ -5821,7 +5838,7 @@
         <v>27</v>
       </c>
       <c r="N71" s="6" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="O71" s="13"/>
       <c r="P71" s="9" t="str">
@@ -5833,18 +5850,18 @@
         <v/>
       </c>
       <c r="R71" s="14" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="4" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B72" s="5" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C72" s="6" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D72" s="7" t="n">
         <v>629</v>
@@ -5858,7 +5875,7 @@
         <v>474</v>
       </c>
       <c r="G72" s="9" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="H72" s="9" t="s">
         <v>153</v>
@@ -5877,7 +5894,7 @@
         <v>27</v>
       </c>
       <c r="N72" s="6" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="O72" s="13"/>
       <c r="P72" s="9" t="str">
@@ -5889,17 +5906,17 @@
         <v/>
       </c>
       <c r="R72" s="14" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="18" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="19" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B75" s="20" t="n">
         <f aca="false">COUNTA(B5:B72)</f>
@@ -5953,7 +5970,7 @@
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="19" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B81" s="20" t="n">
         <f aca="false">COUNTIF($A$5:$A$72,"Постеры")</f>
@@ -5962,7 +5979,7 @@
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="19" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B82" s="20" t="n">
         <f aca="false">COUNTIF(P5:P72,"повтор")</f>
@@ -5971,25 +5988,25 @@
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="19" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B83" s="20" t="n">
         <f aca="false">COUNTIF(Q5:Q72,"дороже лимита")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="19" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B84" s="20" t="n">
         <f aca="false">IFERROR(ROUND(AVERAGE(F5:F72),0),"")</f>
-        <v>700</v>
+        <v>872</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="19" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B85" s="20" t="n">
         <f aca="false">IFERROR(ROUND(AVERAGEIFS(F5:F72,C5:C72,"1:43"),0),"")</f>
@@ -5998,7 +6015,7 @@
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="19" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B86" s="20" t="n">
         <f aca="false">IFERROR(ROUND(AVERAGEIFS(F5:F72,C5:C72,"1:24",A5:A72,"Модели 1:24"),0),"")</f>
@@ -6008,7 +6025,7 @@
   </sheetData>
   <autoFilter ref="A4:R72"/>
   <conditionalFormatting sqref="P5:Q72">
-    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>OR(P5="повтор",Q5="дороже лимита")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6109,39 +6126,39 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="19" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B4" s="21" t="n">
         <v>1500</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="19" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B5" s="22" t="n">
         <v>2</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="19" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B6" s="21" t="n">
         <v>7000</v>
@@ -6150,79 +6167,79 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="19" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B7" s="22" t="n">
         <v>1.6</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="19" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B8" s="22" t="n">
         <v>1.35</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="19" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B9" s="23" t="n">
         <v>0.035</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="19" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="B10" s="23" t="n">
         <v>0.06</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="19" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B11" s="23" t="n">
         <v>0.05</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="19" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B12" s="21" t="n">
         <v>2800</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="19" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B13" s="22" t="n">
         <v>84.2</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
   </sheetData>
@@ -6252,17 +6269,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="24" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B4" s="24" t="s">
         <v>6</v>
@@ -6274,12 +6291,12 @@
         <v>8</v>
       </c>
       <c r="E4" s="24" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="19" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B5" s="21" t="n">
         <v>289</v>
@@ -6296,7 +6313,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="19" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B6" s="21" t="n">
         <v>379</v>
@@ -6313,7 +6330,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="19" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B7" s="21" t="n">
         <v>472</v>
@@ -6330,7 +6347,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="19" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B8" s="21" t="n">
         <v>519</v>
@@ -6344,12 +6361,12 @@
         <v>413</v>
       </c>
       <c r="E8" s="26" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="19" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B9" s="21" t="n">
         <v>629</v>
@@ -6363,12 +6380,12 @@
         <v>474</v>
       </c>
       <c r="E9" s="26" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="19" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B10" s="21" t="n">
         <v>829</v>
@@ -6385,7 +6402,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="19" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B11" s="21" t="n">
         <v>931</v>
@@ -6399,12 +6416,12 @@
         <v>685</v>
       </c>
       <c r="E11" s="26" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="19" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B12" s="21" t="n">
         <v>1052</v>
@@ -6418,12 +6435,12 @@
         <v>820</v>
       </c>
       <c r="E12" s="26" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="19" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B13" s="21" t="n">
         <v>1269</v>
@@ -6440,7 +6457,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="19" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B14" s="21" t="n">
         <v>1372</v>
@@ -6457,175 +6474,175 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="18" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="26" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B17" s="19" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="26" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B18" s="19" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="26" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B19" s="19" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="26" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B20" s="19" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="26" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B21" s="19" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="26" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B22" s="19" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="26" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="B23" s="19" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="26" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B24" s="19" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="26" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B25" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="26" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B26" s="19" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="26" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="B27" s="19" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="26" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B28" s="19" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="26" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B29" s="19" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="26" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B30" s="19" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="26" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="B31" s="19" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="26" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B32" s="19" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="26" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B33" s="19" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="26" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B34" s="19" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="26" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="B35" s="19" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="26" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B36" s="19" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="26" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B37" s="19" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
     </row>
   </sheetData>
@@ -6660,12 +6677,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6691,21 +6708,21 @@
         <v>5</v>
       </c>
       <c r="H4" s="24" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="I4" s="24" t="s">
         <v>14</v>
       </c>
       <c r="J4" s="24" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="K4" s="24" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="27" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="B5" s="28" t="s">
         <v>39</v>
@@ -6729,18 +6746,18 @@
         <v>789</v>
       </c>
       <c r="I5" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J5" s="28" t="n">
         <v>1947</v>
       </c>
       <c r="K5" s="30" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="27" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="B6" s="28" t="s">
         <v>33</v>
@@ -6764,18 +6781,18 @@
         <v>789</v>
       </c>
       <c r="I6" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J6" s="28" t="n">
         <v>1947</v>
       </c>
       <c r="K6" s="30" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="27" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="B7" s="28" t="s">
         <v>28</v>
@@ -6799,18 +6816,18 @@
         <v>789</v>
       </c>
       <c r="I7" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J7" s="28" t="n">
         <v>1947</v>
       </c>
       <c r="K7" s="30" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="27" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="B8" s="28" t="s">
         <v>51</v>
@@ -6834,18 +6851,18 @@
         <v>789</v>
       </c>
       <c r="I8" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J8" s="28" t="n">
         <v>1947</v>
       </c>
       <c r="K8" s="30" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="27" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="B9" s="28" t="s">
         <v>76</v>
@@ -6869,18 +6886,18 @@
         <v>789</v>
       </c>
       <c r="I9" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J9" s="28" t="n">
         <v>1947</v>
       </c>
       <c r="K9" s="30" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="27" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="B10" s="28" t="s">
         <v>64</v>
@@ -6904,18 +6921,18 @@
         <v>789</v>
       </c>
       <c r="I10" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J10" s="28" t="n">
         <v>1947</v>
       </c>
       <c r="K10" s="30" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="27" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="B11" s="28" t="s">
         <v>53</v>
@@ -6939,18 +6956,18 @@
         <v>789</v>
       </c>
       <c r="I11" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J11" s="28" t="n">
         <v>1947</v>
       </c>
       <c r="K11" s="30" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="27" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="B12" s="28" t="s">
         <v>47</v>
@@ -6974,18 +6991,18 @@
         <v>789</v>
       </c>
       <c r="I12" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J12" s="28" t="n">
         <v>1947</v>
       </c>
       <c r="K12" s="30" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="27" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="B13" s="28" t="s">
         <v>73</v>
@@ -7009,18 +7026,18 @@
         <v>789</v>
       </c>
       <c r="I13" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J13" s="28" t="n">
         <v>1947</v>
       </c>
       <c r="K13" s="30" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="27" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="B14" s="28" t="s">
         <v>78</v>
@@ -7044,18 +7061,18 @@
         <v>789</v>
       </c>
       <c r="I14" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J14" s="28" t="n">
         <v>1947</v>
       </c>
       <c r="K14" s="30" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="27" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="B15" s="28" t="s">
         <v>67</v>
@@ -7079,21 +7096,21 @@
         <v>789</v>
       </c>
       <c r="I15" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J15" s="28" t="n">
         <v>1947</v>
       </c>
       <c r="K15" s="30" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="27" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B16" s="28" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C16" s="28" t="s">
         <v>41</v>
@@ -7114,18 +7131,18 @@
         <v>879</v>
       </c>
       <c r="I16" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J16" s="28" t="n">
         <v>791</v>
       </c>
       <c r="K16" s="28" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="27" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B17" s="28" t="s">
         <v>44</v>
@@ -7149,21 +7166,21 @@
         <v>879</v>
       </c>
       <c r="I17" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J17" s="28" t="n">
         <v>791</v>
       </c>
       <c r="K17" s="30" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="27" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B18" s="28" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="C18" s="28" t="s">
         <v>41</v>
@@ -7184,21 +7201,21 @@
         <v>879</v>
       </c>
       <c r="I18" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J18" s="28" t="n">
         <v>791</v>
       </c>
       <c r="K18" s="28" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="27" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B19" s="28" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="C19" s="28" t="s">
         <v>24</v>
@@ -7219,21 +7236,21 @@
         <v>879</v>
       </c>
       <c r="I19" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J19" s="28" t="n">
         <v>791</v>
       </c>
       <c r="K19" s="28" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="27" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B20" s="28" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="C20" s="28" t="s">
         <v>24</v>
@@ -7254,18 +7271,18 @@
         <v>879</v>
       </c>
       <c r="I20" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J20" s="28" t="n">
         <v>791</v>
       </c>
       <c r="K20" s="28" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="27" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B21" s="28" t="s">
         <v>37</v>
@@ -7289,21 +7306,21 @@
         <v>879</v>
       </c>
       <c r="I21" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J21" s="28" t="n">
         <v>791</v>
       </c>
       <c r="K21" s="30" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="27" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B22" s="28" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C22" s="28" t="s">
         <v>24</v>
@@ -7324,18 +7341,18 @@
         <v>879</v>
       </c>
       <c r="I22" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J22" s="28" t="n">
         <v>791</v>
       </c>
       <c r="K22" s="28" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="27" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B23" s="28" t="s">
         <v>57</v>
@@ -7359,21 +7376,21 @@
         <v>879</v>
       </c>
       <c r="I23" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J23" s="28" t="n">
         <v>791</v>
       </c>
       <c r="K23" s="30" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="27" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B24" s="28" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C24" s="28" t="s">
         <v>55</v>
@@ -7394,18 +7411,18 @@
         <v>879</v>
       </c>
       <c r="I24" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J24" s="28" t="n">
         <v>791</v>
       </c>
       <c r="K24" s="28" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="27" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B25" s="28" t="s">
         <v>71</v>
@@ -7429,21 +7446,21 @@
         <v>879</v>
       </c>
       <c r="I25" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J25" s="28" t="n">
         <v>791</v>
       </c>
       <c r="K25" s="30" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="27" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B26" s="28" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="C26" s="28" t="s">
         <v>69</v>
@@ -7464,18 +7481,18 @@
         <v>879</v>
       </c>
       <c r="I26" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J26" s="28" t="n">
         <v>791</v>
       </c>
       <c r="K26" s="28" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="27" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B27" s="28" t="s">
         <v>82</v>
@@ -7499,18 +7516,18 @@
         <v>879</v>
       </c>
       <c r="I27" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J27" s="28" t="n">
         <v>791</v>
       </c>
       <c r="K27" s="30" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="27" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B28" s="28" t="s">
         <v>85</v>
@@ -7534,18 +7551,18 @@
         <v>879</v>
       </c>
       <c r="I28" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J28" s="28" t="n">
         <v>791</v>
       </c>
       <c r="K28" s="30" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="27" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B29" s="28" t="s">
         <v>94</v>
@@ -7569,18 +7586,18 @@
         <v>879</v>
       </c>
       <c r="I29" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J29" s="28" t="n">
         <v>791</v>
       </c>
       <c r="K29" s="30" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="27" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B30" s="28" t="s">
         <v>90</v>
@@ -7604,21 +7621,21 @@
         <v>879</v>
       </c>
       <c r="I30" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J30" s="28" t="n">
         <v>791</v>
       </c>
       <c r="K30" s="30" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="27" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B31" s="28" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="C31" s="28" t="s">
         <v>69</v>
@@ -7639,18 +7656,18 @@
         <v>879</v>
       </c>
       <c r="I31" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J31" s="28" t="n">
         <v>791</v>
       </c>
       <c r="K31" s="28" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="27" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B32" s="28" t="s">
         <v>60</v>
@@ -7674,21 +7691,21 @@
         <v>879</v>
       </c>
       <c r="I32" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J32" s="28" t="n">
         <v>791</v>
       </c>
       <c r="K32" s="30" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="27" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B33" s="28" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="C33" s="28" t="s">
         <v>55</v>
@@ -7709,21 +7726,21 @@
         <v>879</v>
       </c>
       <c r="I33" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J33" s="28" t="n">
         <v>791</v>
       </c>
       <c r="K33" s="28" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="27" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B34" s="28" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C34" s="28" t="s">
         <v>69</v>
@@ -7744,18 +7761,18 @@
         <v>879</v>
       </c>
       <c r="I34" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J34" s="28" t="n">
         <v>791</v>
       </c>
       <c r="K34" s="28" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="27" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="B35" s="28" t="s">
         <v>101</v>
@@ -7779,18 +7796,18 @@
         <v>1489</v>
       </c>
       <c r="I35" s="28" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="J35" s="28" t="n">
         <v>45</v>
       </c>
       <c r="K35" s="30" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="27" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="B36" s="28" t="s">
         <v>98</v>
@@ -7814,18 +7831,18 @@
         <v>1489</v>
       </c>
       <c r="I36" s="28" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="J36" s="28" t="n">
         <v>45</v>
       </c>
       <c r="K36" s="30" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="27" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="B37" s="28" t="s">
         <v>104</v>
@@ -7849,18 +7866,18 @@
         <v>1489</v>
       </c>
       <c r="I37" s="28" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="J37" s="28" t="n">
         <v>31</v>
       </c>
       <c r="K37" s="30" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="27" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="B38" s="28" t="s">
         <v>106</v>
@@ -7884,18 +7901,18 @@
         <v>1489</v>
       </c>
       <c r="I38" s="28" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="J38" s="28" t="n">
         <v>31</v>
       </c>
       <c r="K38" s="30" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="27" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B39" s="28" t="s">
         <v>112</v>
@@ -7919,18 +7936,18 @@
         <v>2682</v>
       </c>
       <c r="I39" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J39" s="28" t="n">
         <v>653</v>
       </c>
       <c r="K39" s="30" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="27" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B40" s="28" t="s">
         <v>120</v>
@@ -7954,18 +7971,18 @@
         <v>2659</v>
       </c>
       <c r="I40" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J40" s="28" t="n">
         <v>653</v>
       </c>
       <c r="K40" s="28" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="27" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B41" s="28" t="s">
         <v>117</v>
@@ -7989,18 +8006,18 @@
         <v>2439</v>
       </c>
       <c r="I41" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J41" s="28" t="n">
         <v>653</v>
       </c>
       <c r="K41" s="28" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="27" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B42" s="28" t="s">
         <v>135</v>
@@ -8024,18 +8041,18 @@
         <v>2649</v>
       </c>
       <c r="I42" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J42" s="28" t="n">
         <v>653</v>
       </c>
       <c r="K42" s="28" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="27" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B43" s="28" t="s">
         <v>128</v>
@@ -8059,18 +8076,18 @@
         <v>2679</v>
       </c>
       <c r="I43" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J43" s="28" t="n">
         <v>653</v>
       </c>
       <c r="K43" s="30" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="27" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B44" s="28" t="s">
         <v>149</v>
@@ -8094,18 +8111,18 @@
         <v>2430</v>
       </c>
       <c r="I44" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J44" s="28" t="n">
         <v>653</v>
       </c>
       <c r="K44" s="28" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="27" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B45" s="28" t="s">
         <v>124</v>
@@ -8129,18 +8146,18 @@
         <v>2461</v>
       </c>
       <c r="I45" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J45" s="28" t="n">
         <v>653</v>
       </c>
       <c r="K45" s="28" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="27" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B46" s="28" t="s">
         <v>145</v>
@@ -8164,18 +8181,18 @@
         <v>2549</v>
       </c>
       <c r="I46" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J46" s="28" t="n">
         <v>651</v>
       </c>
       <c r="K46" s="30" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="27" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B47" s="28" t="s">
         <v>120</v>
@@ -8199,18 +8216,18 @@
         <v>2522</v>
       </c>
       <c r="I47" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J47" s="28" t="n">
         <v>651</v>
       </c>
       <c r="K47" s="28" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="27" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B48" s="28" t="s">
         <v>117</v>
@@ -8234,18 +8251,18 @@
         <v>2312</v>
       </c>
       <c r="I48" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J48" s="28" t="n">
         <v>651</v>
       </c>
       <c r="K48" s="30" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="27" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B49" s="28" t="s">
         <v>138</v>
@@ -8269,18 +8286,18 @@
         <v>2509</v>
       </c>
       <c r="I49" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J49" s="28" t="n">
         <v>651</v>
       </c>
       <c r="K49" s="30" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="27" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B50" s="28" t="s">
         <v>135</v>
@@ -8304,18 +8321,18 @@
         <v>2509</v>
       </c>
       <c r="I50" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J50" s="28" t="n">
         <v>651</v>
       </c>
       <c r="K50" s="30" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="27" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B51" s="28" t="s">
         <v>124</v>
@@ -8339,18 +8356,18 @@
         <v>2542</v>
       </c>
       <c r="I51" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J51" s="28" t="n">
         <v>651</v>
       </c>
       <c r="K51" s="28" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="27" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B52" s="28" t="s">
         <v>149</v>
@@ -8374,18 +8391,18 @@
         <v>2522</v>
       </c>
       <c r="I52" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J52" s="28" t="n">
         <v>651</v>
       </c>
       <c r="K52" s="28" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="27" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B53" s="28" t="s">
         <v>142</v>
@@ -8409,18 +8426,18 @@
         <v>2092</v>
       </c>
       <c r="I53" s="28" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="J53" s="28" t="n">
         <v>45</v>
       </c>
       <c r="K53" s="30" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="27" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B54" s="28" t="s">
         <v>147</v>
@@ -8444,18 +8461,18 @@
         <v>2092</v>
       </c>
       <c r="I54" s="28" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="J54" s="28" t="n">
         <v>45</v>
       </c>
       <c r="K54" s="30" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="27" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B55" s="28" t="s">
         <v>117</v>
@@ -8479,18 +8496,18 @@
         <v>2409</v>
       </c>
       <c r="I55" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J55" s="28" t="n">
         <v>78</v>
       </c>
       <c r="K55" s="28" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="27" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B56" s="28" t="s">
         <v>120</v>
@@ -8514,18 +8531,18 @@
         <v>2409</v>
       </c>
       <c r="I56" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J56" s="28" t="n">
         <v>78</v>
       </c>
       <c r="K56" s="30" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="27" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B57" s="28" t="s">
         <v>135</v>
@@ -8549,18 +8566,18 @@
         <v>2611</v>
       </c>
       <c r="I57" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J57" s="28" t="n">
         <v>78</v>
       </c>
       <c r="K57" s="28" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="27" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B58" s="28" t="s">
         <v>124</v>
@@ -8584,18 +8601,18 @@
         <v>2421</v>
       </c>
       <c r="I58" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J58" s="28" t="n">
         <v>78</v>
       </c>
       <c r="K58" s="30" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="27" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B59" s="28" t="s">
         <v>148</v>
@@ -8619,18 +8636,18 @@
         <v>2631</v>
       </c>
       <c r="I59" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J59" s="28" t="n">
         <v>78</v>
       </c>
       <c r="K59" s="30" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="27" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B60" s="28" t="s">
         <v>149</v>
@@ -8654,18 +8671,18 @@
         <v>2401</v>
       </c>
       <c r="I60" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J60" s="28" t="n">
         <v>78</v>
       </c>
       <c r="K60" s="30" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="27" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B61" s="28" t="s">
         <v>132</v>
@@ -8689,13 +8706,13 @@
         <v>2439</v>
       </c>
       <c r="I61" s="28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J61" s="28" t="n">
         <v>78</v>
       </c>
       <c r="K61" s="30" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
   </sheetData>
@@ -8784,95 +8801,95 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="31" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B3" s="32" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="31" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="B4" s="32" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="31" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="B5" s="32" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="31" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B6" s="32" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="31" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="B7" s="32" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="31" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="B8" s="32" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="31" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="B9" s="32" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="31" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="B10" s="32" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="31" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="B11" s="32" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="31" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="B12" s="32" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="31" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B13" s="32" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
     </row>
   </sheetData>

</xml_diff>